<commit_message>
Omit disconnected nodes from the rendered flow diagram
Tables declared as a SOURCE/TARGET in the file but never actually wired
into a mapping (e.g. an unused lookup source) were showing up as
disconnected boxes in the Flow Diagram sheet. A flowchart should only
show things that actually flow, so these are filtered out; the Table/
Column Lineage sheets were unaffected since they only ever listed edges.
Also add docs/images/ with standalone copies of the two sample diagrams
for use in written material about the project.
</commit_message>
<xml_diff>
--- a/output/sample_banking_dw_lineage_mapping.xlsx
+++ b/output/sample_banking_dw_lineage_mapping.xlsx
@@ -148,7 +148,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7515225" cy="2209800"/>
+    <ext cx="7515225" cy="2009775"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -790,7 +790,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>total_deposits_usd</t>
+          <t>total_withdrawals_usd</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>total_withdrawals_usd</t>
+          <t>total_deposits_usd</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>total_deposits_usd</t>
+          <t>total_withdrawals_usd</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>total_withdrawals_usd</t>
+          <t>total_deposits_usd</t>
         </is>
       </c>
     </row>

</xml_diff>